<commit_message>
update ngay den han
</commit_message>
<xml_diff>
--- a/templates/template_bmk_ngay_dao_han.xlsx
+++ b/templates/template_bmk_ngay_dao_han.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\programme\git_repository\bmk\bmk-ctv-service\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69BF71F6-72C1-4631-A562-F425E3F5DECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCA8CCC-B13C-433B-ADFC-20CBDD0E48B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="CTV ngày đáo hạn" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CTV ngày đáo hạn'!$A$3:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CTV ngày đáo hạn'!$A$3:$D$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Số lượng:</t>
   </si>
@@ -40,24 +40,6 @@
     <t>Số CCCD</t>
   </si>
   <si>
-    <t>ĐÃ LÀM</t>
-  </si>
-  <si>
-    <t>THUẾ</t>
-  </si>
-  <si>
-    <t>BHXH</t>
-  </si>
-  <si>
-    <t>check chênh lệchh</t>
-  </si>
-  <si>
-    <t>chênh lệch</t>
-  </si>
-  <si>
-    <t>FILE</t>
-  </si>
-  <si>
     <t>06977</t>
   </si>
   <si>
@@ -67,23 +49,20 @@
     <t>001089000788</t>
   </si>
   <si>
-    <t>Hiện diện đã làm</t>
-  </si>
-  <si>
-    <t>HIỆN DIỆN</t>
-  </si>
-  <si>
     <t>DANH SÁCH CẬP NHẬT NGÀY ĐÁO HẠN HỢP ĐỒNG</t>
   </si>
   <si>
     <t>Ngày đáo hạn</t>
+  </si>
+  <si>
+    <t>Ngày gia nhập</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -124,21 +103,8 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,24 +119,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
-        <bgColor rgb="FF7030A0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor theme="0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -205,13 +159,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -226,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -237,13 +184,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -256,28 +196,16 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -507,115 +435,74 @@
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.54296875" customWidth="1"/>
     <col min="2" max="2" width="13.453125" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="16.7265625" customWidth="1"/>
-    <col min="5" max="5" width="27.1796875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="16.453125" hidden="1" customWidth="1"/>
-    <col min="8" max="9" width="11.81640625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="16" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="17" style="19" customWidth="1"/>
+    <col min="5" max="5" width="17" style="12" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="5">
         <v>1</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:6" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="C4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
-        <v>1</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" s="19">
+      <c r="E4" s="12">
         <v>46346</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
   <headerFooter>

</xml_diff>